<commit_message>
feat(pageObjects): Add CartPage and update MyAccountPage locators
- Introduces a new `CartPage` object for interacting with the shopping cart.
- Adds locators and methods for checking cart display, product presence, removing items, and verifying an empty cart.
- Updates `MyAccountPage` with new locators for menu items and links.
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eclipse-workspace\OpenCartFramework\testData\"/>
     </mc:Choice>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="52">
   <si>
     <t>TestCase</t>
   </si>
@@ -177,12 +177,19 @@
   </si>
   <si>
     <t>qwertyuiop</t>
+  </si>
+  <si>
+    <t>test1779587740008@gmail.com</t>
+  </si>
+  <si>
+    <t>test1779594809649@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -532,10 +539,10 @@
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="17.28515625"/>
+    <col min="2" max="2" customWidth="true" width="20.28515625"/>
+    <col min="3" max="3" customWidth="true" width="20.5703125"/>
+    <col min="4" max="4" customWidth="true" width="18.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -553,16 +560,16 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>27</v>
       </c>
     </row>
@@ -656,9 +663,9 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.28515625" customWidth="1"/>
-    <col min="2" max="2" width="37.85546875" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="36.28515625"/>
+    <col min="2" max="2" customWidth="true" width="37.85546875"/>
+    <col min="3" max="3" customWidth="true" width="16.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -792,12 +799,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="26.42578125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="18.42578125"/>
+    <col min="2" max="2" customWidth="true" width="19.42578125"/>
+    <col min="3" max="3" customWidth="true" width="18.42578125"/>
+    <col min="4" max="4" customWidth="true" width="21.0"/>
+    <col min="5" max="5" customWidth="true" width="15.7109375"/>
+    <col min="6" max="6" customWidth="true" width="26.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -821,22 +828,22 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="C2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="D2" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(lighthouse): Add OpenCart Lighthouse report
- Includes the generated HTML report for Lighthouse analysis.
- This report provides insights into the performance and accessibility of the OpenCart site.
- Facilitates performance optimization efforts.
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eclipse-workspace\OpenCartFramework\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8519D146-2423-4BB7-9908-BDF515B58666}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35CE3B4C-7B87-4B82-A292-076A4F298CA5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="50">
   <si>
     <t>TestCase</t>
   </si>
@@ -113,9 +113,6 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>test1779587041213@gmail.com</t>
-  </si>
-  <si>
     <t>SearchText</t>
   </si>
   <si>
@@ -177,9 +174,6 @@
   </si>
   <si>
     <t>qwertyuiop</t>
-  </si>
-  <si>
-    <t>test1779587740008@gmail.com</t>
   </si>
   <si>
     <t>test1779594809649@gmail.com</t>
@@ -189,7 +183,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -539,10 +532,10 @@
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="17.28515625"/>
-    <col min="2" max="2" customWidth="true" width="20.28515625"/>
-    <col min="3" max="3" customWidth="true" width="20.5703125"/>
-    <col min="4" max="4" customWidth="true" width="18.7109375"/>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -560,16 +553,16 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="C2" t="s" s="0">
+      <c r="B2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>27</v>
       </c>
     </row>
@@ -663,9 +656,9 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="36.28515625"/>
-    <col min="2" max="2" customWidth="true" width="37.85546875"/>
-    <col min="3" max="3" customWidth="true" width="16.140625"/>
+    <col min="1" max="1" width="36.28515625" customWidth="1"/>
+    <col min="2" max="2" width="37.85546875" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -673,7 +666,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>3</v>
@@ -681,10 +674,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -692,10 +685,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -703,10 +696,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
@@ -714,10 +707,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
@@ -725,10 +718,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>6</v>
@@ -736,10 +729,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>10</v>
@@ -747,10 +740,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>10</v>
@@ -758,10 +751,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>10</v>
@@ -769,10 +762,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>10</v>
@@ -780,10 +773,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>10</v>
@@ -799,12 +792,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="18.42578125"/>
-    <col min="2" max="2" customWidth="true" width="19.42578125"/>
-    <col min="3" max="3" customWidth="true" width="18.42578125"/>
-    <col min="4" max="4" customWidth="true" width="21.0"/>
-    <col min="5" max="5" customWidth="true" width="15.7109375"/>
-    <col min="6" max="6" customWidth="true" width="26.42578125"/>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="4" max="4" width="21" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -828,22 +821,22 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>25</v>
       </c>
-      <c r="C2" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="D2" t="s" s="0">
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s">
         <v>26</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(performance): Add JMeter tests for OpenCart performance
- Introduces JMeter test plans for homepage load, login stress, and search performance.
- Includes page object models and test cases for various user flows.
- Updates test data and configuration files.
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eclipse-workspace\OpenCartFramework\testData\"/>
     </mc:Choice>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="53">
   <si>
     <t>TestCase</t>
   </si>
@@ -177,12 +177,22 @@
   </si>
   <si>
     <t>test1779594809649@gmail.com</t>
+  </si>
+  <si>
+    <t>test1779828712469@gmail.com</t>
+  </si>
+  <si>
+    <t>test1779837428810@gmail.com</t>
+  </si>
+  <si>
+    <t>test1779838137948@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -532,10 +542,10 @@
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="17.28515625"/>
+    <col min="2" max="2" customWidth="true" width="20.28515625"/>
+    <col min="3" max="3" customWidth="true" width="20.5703125"/>
+    <col min="4" max="4" customWidth="true" width="18.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -553,16 +563,16 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>27</v>
       </c>
     </row>
@@ -656,9 +666,9 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.28515625" customWidth="1"/>
-    <col min="2" max="2" width="37.85546875" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="36.28515625"/>
+    <col min="2" max="2" customWidth="true" width="37.85546875"/>
+    <col min="3" max="3" customWidth="true" width="16.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -792,12 +802,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
-    <col min="4" max="4" width="21" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="26.42578125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="18.42578125"/>
+    <col min="2" max="2" customWidth="true" width="19.42578125"/>
+    <col min="3" max="3" customWidth="true" width="18.42578125"/>
+    <col min="4" max="4" customWidth="true" width="21.0"/>
+    <col min="5" max="5" customWidth="true" width="15.7109375"/>
+    <col min="6" max="6" customWidth="true" width="26.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -821,22 +831,22 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="C2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="D2" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
test(AccountRegistration): Improve logging and data persistence for registration
- Enhanced logging to provide clearer step-by-step execution and success indicators.
- Integrated writing of registered user data (email, password) to both 'RegisterData' and 'LoginData' sheets in TestData.xlsx.
- Added explicit logging for Excel operations and data generation.
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="56">
   <si>
     <t>TestCase</t>
   </si>
@@ -186,6 +186,15 @@
   </si>
   <si>
     <t>test1779838137948@gmail.com</t>
+  </si>
+  <si>
+    <t>test1780017314212@gmail.com</t>
+  </si>
+  <si>
+    <t>test1780017359057@gmail.com</t>
+  </si>
+  <si>
+    <t>test1780020856078@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -567,7 +576,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>5</v>
@@ -838,7 +847,7 @@
         <v>25</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>5</v>

</xml_diff>

<commit_message>
feat(base): Integrate Selenium Grid for remote execution
- Modified `setup` method to accept `runMode` parameter.
- Implemented logic to launch browsers via Selenium Grid when `runMode` is 'grid'.
- Added support for Chrome, Firefox, and Edge on the grid.
- Included necessary imports for `URL`, `ChromeOptions`, `FirefoxOptions`, `EdgeOptions`, and `RemoteWebDriver`.
</commit_message>
<xml_diff>
--- a/testData/TestData.xlsx
+++ b/testData/TestData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="59">
   <si>
     <t>TestCase</t>
   </si>
@@ -195,6 +195,15 @@
   </si>
   <si>
     <t>test1780020856078@gmail.com</t>
+  </si>
+  <si>
+    <t>test1781383464613@gmail.com</t>
+  </si>
+  <si>
+    <t>test1781384004434@gmail.com</t>
+  </si>
+  <si>
+    <t>test1781386426052@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -576,7 +585,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s" s="0">
         <v>5</v>
@@ -847,7 +856,7 @@
         <v>25</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>5</v>

</xml_diff>